<commit_message>
v1.11.0: código de venta automático + proveedor en insumos
Calcula el código de venta automáticamente a partir de las iniciales
de la clienta y la fecha del evento (DDMMYY), tanto al crear una venta
a mano (sugerido y editable, con botón para recalcular) como al aceptar
una cotización (reemplaza el esquema anterior COT-xxxxxx). Resuelve
colisiones agregando un sufijo automático para garantizar unicidad.

Agrega un campo opcional "Proveedor" al Registro de insumos, en la app
y en la plantilla Excel de importación.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GYzn3WtyZgSGWpLH2sAFg9
</commit_message>
<xml_diff>
--- a/client/public/plantilla-compras.xlsx
+++ b/client/public/plantilla-compras.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
   <si>
     <t>FECHA COMPRA</t>
   </si>
@@ -20,6 +20,9 @@
     <t>CATEGORIA</t>
   </si>
   <si>
+    <t>PROVEEDOR</t>
+  </si>
+  <si>
     <t>DESCRIPCION</t>
   </si>
   <si>
@@ -35,6 +38,9 @@
     <t>Encaje / Adorno</t>
   </si>
   <si>
+    <t>Telas Hermanos Soto</t>
+  </si>
+  <si>
     <t>Encaje francés para vestido de Josefina</t>
   </si>
   <si>
@@ -90,6 +96,9 @@
   </si>
   <si>
     <t>Tela, Forro, Encaje / Adorno, Cierre / Botones, Hilos / Agujas / Alfileres u Otros materiales (lista desplegable).</t>
+  </si>
+  <si>
+    <t>Nombre del proveedor o tienda (opcional).</t>
   </si>
   <si>
     <t>Qué se compró, en tus palabras. Ej: 'Tul bordado premium'.</t>
@@ -120,9 +129,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -133,19 +139,19 @@
     </font>
     <font>
       <b/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
-      <color rgb="008A7F75"/>
+      <color rgb="FF8A7F75"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <color rgb="00C9A96E"/>
+      <color rgb="FFC9A96E"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -159,7 +165,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A1A2E"/>
+        <fgColor rgb="FF1A1A2E"/>
       </patternFill>
     </fill>
   </fills>
@@ -177,10 +183,8 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -522,19 +526,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="60" customWidth="1"/>
+    <col min="2" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -553,121 +557,61 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>46178</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="3">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3">
         <v>150000</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="F2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>46179</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="3">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="3">
         <v>60000</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="2:5" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:5" x14ac:dyDescent="0.25"/>
+      <c r="F3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" s="3"/>
+    </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" errorTitle="Categoría inválida" error="Elige una categoría de la lista." sqref="B10:B64">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" errorTitle="Categoría inválida" error="Elige una categoría de la lista." sqref="B2:B3">
       <formula1>"Tela,Forro,Encaje / Adorno,Cierre / Botones,Hilos / Agujas / Alfileres,Otros materiales"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorTitle="Categoría inválida" error="Elige una categoría de la lista." sqref="B2:B64">
-      <formula1>"Tela,Forro,Encaje / Adorno,Cierre / Botones,Hilos / Agujas / Alfileres,Otros materiales"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorTitle="Tipo de asignación inválido" error="Elige un tipo de asignación de la lista." sqref="E10:E64">
-      <formula1>"Directo,Prorrateo"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorTitle="Tipo de asignación inválido" error="Elige un tipo de asignación de la lista." sqref="E2:E64">
+    <dataValidation type="list" allowBlank="1" errorTitle="Tipo de asignación inválido" error="Elige un tipo de asignación de la lista." sqref="F2:F3">
       <formula1>"Directo,Prorrateo"</formula1>
     </dataValidation>
   </dataValidations>
@@ -678,7 +622,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -687,55 +631,65 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5"/>
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6"/>
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7"/>
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8"/>
+        <v>22</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9"/>
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -743,7 +697,7 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -751,7 +705,7 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -759,7 +713,7 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -767,7 +721,7 @@
         <v>3</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -775,7 +729,7 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -783,45 +737,47 @@
         <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>8</v>
-      </c>
-      <c r="B20" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B21" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A23:B23"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>